<commit_message>
Add final planform and sector-envelope supplementary package
</commit_message>
<xml_diff>
--- a/Source_Data/Supplementary_Tables.xlsx
+++ b/Source_Data/Supplementary_Tables.xlsx
@@ -25,8 +25,11 @@
     <sheet name="21_table_s_energy_emissions_gri" sheetId="21" r:id="rId21"/>
     <sheet name="22_table_s_external_calibration" sheetId="22" r:id="rId22"/>
     <sheet name="23_table_s_external_pv_calibrat" sheetId="23" r:id="rId23"/>
-    <sheet name="24_table_s_segment_economic_res" sheetId="24" r:id="rId24"/>
-    <sheet name="25_table_s_urban_evidence_bound" sheetId="25" r:id="rId25"/>
+    <sheet name="24_table_s_planform_local_conte" sheetId="24" r:id="rId24"/>
+    <sheet name="25_table_s_planform_local_conte" sheetId="25" r:id="rId25"/>
+    <sheet name="26_table_s_sector_economic_enve" sheetId="26" r:id="rId26"/>
+    <sheet name="27_table_s_segment_economic_res" sheetId="27" r:id="rId27"/>
+    <sheet name="28_table_s_urban_evidence_bound" sheetId="28" r:id="rId28"/>
   </sheets>
 </workbook>
 </file>
@@ -6563,6 +6566,3840 @@
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:N13"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">outcome</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">feature</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">feature_label</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">coefficient</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">multiplicative_effect_per_sd</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">model_metric_name</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">model_metric</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">sample_size</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">city_model_count</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">city_positive_effect_count</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">city_negative_effect_count</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">city_effect_median</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">city_effect_min</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">city_effect_max</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PV-positive prevalence</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">log_footprint_area</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Footprint area</t>
+        </is>
+      </c>
+      <c r="D2">
+        <v>1.2422523456096577</v>
+      </c>
+      <c r="E2">
+        <v>3.463405472431729</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">weighted ROC AUC</t>
+        </is>
+      </c>
+      <c r="G2">
+        <v>0.8410124478746281</v>
+      </c>
+      <c r="H2">
+        <v>686095</v>
+      </c>
+      <c r="I2">
+        <v>11</v>
+      </c>
+      <c r="J2">
+        <v>11</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>3.182339919745728</v>
+      </c>
+      <c r="M2">
+        <v>2.3206052175030925</v>
+      </c>
+      <c r="N2">
+        <v>5.401517423096429</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PV-positive prevalence</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">compactness</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Planform compactness</t>
+        </is>
+      </c>
+      <c r="D3">
+        <v>0.005085161607756525</v>
+      </c>
+      <c r="E3">
+        <v>1.0050981129860228</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">weighted ROC AUC</t>
+        </is>
+      </c>
+      <c r="G3">
+        <v>0.8410124478746281</v>
+      </c>
+      <c r="H3">
+        <v>686095</v>
+      </c>
+      <c r="I3">
+        <v>11</v>
+      </c>
+      <c r="J3">
+        <v>5</v>
+      </c>
+      <c r="K3">
+        <v>6</v>
+      </c>
+      <c r="L3">
+        <v>0.9955278497936506</v>
+      </c>
+      <c r="M3">
+        <v>0.8589791950791544</v>
+      </c>
+      <c r="N3">
+        <v>1.3001783473130972</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PV-positive prevalence</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">log_elongation</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Planform elongation</t>
+        </is>
+      </c>
+      <c r="D4">
+        <v>-0.14779993226699256</v>
+      </c>
+      <c r="E4">
+        <v>0.8626036768415454</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">weighted ROC AUC</t>
+        </is>
+      </c>
+      <c r="G4">
+        <v>0.8410124478746281</v>
+      </c>
+      <c r="H4">
+        <v>686095</v>
+      </c>
+      <c r="I4">
+        <v>11</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4">
+        <v>10</v>
+      </c>
+      <c r="L4">
+        <v>0.8609891786134595</v>
+      </c>
+      <c r="M4">
+        <v>0.7475727103730135</v>
+      </c>
+      <c r="N4">
+        <v>1.0839562637304472</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PV-positive prevalence</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cardinal_alignment</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cardinal-axis alignment</t>
+        </is>
+      </c>
+      <c r="D5">
+        <v>0.010818679973225366</v>
+      </c>
+      <c r="E5">
+        <v>1.010877413506748</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">weighted ROC AUC</t>
+        </is>
+      </c>
+      <c r="G5">
+        <v>0.8410124478746281</v>
+      </c>
+      <c r="H5">
+        <v>686095</v>
+      </c>
+      <c r="I5">
+        <v>11</v>
+      </c>
+      <c r="J5">
+        <v>7</v>
+      </c>
+      <c r="K5">
+        <v>4</v>
+      </c>
+      <c r="L5">
+        <v>1.059401934059581</v>
+      </c>
+      <c r="M5">
+        <v>0.8664695540258964</v>
+      </c>
+      <c r="N5">
+        <v>1.171761490972158</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PV-positive prevalence</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">log_local_building_density</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Local building density</t>
+        </is>
+      </c>
+      <c r="D6">
+        <v>0.17071332989140775</v>
+      </c>
+      <c r="E6">
+        <v>1.1861506663379449</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">weighted ROC AUC</t>
+        </is>
+      </c>
+      <c r="G6">
+        <v>0.8410124478746281</v>
+      </c>
+      <c r="H6">
+        <v>686095</v>
+      </c>
+      <c r="I6">
+        <v>11</v>
+      </c>
+      <c r="J6">
+        <v>6</v>
+      </c>
+      <c r="K6">
+        <v>5</v>
+      </c>
+      <c r="L6">
+        <v>1.0179880346814523</v>
+      </c>
+      <c r="M6">
+        <v>0.5091020676818024</v>
+      </c>
+      <c r="N6">
+        <v>1.6283484010802955</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PV-positive prevalence</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">log_local_footprint_coverage</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Local footprint coverage</t>
+        </is>
+      </c>
+      <c r="D7">
+        <v>-0.2854500424128218</v>
+      </c>
+      <c r="E7">
+        <v>0.7516758921542659</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">weighted ROC AUC</t>
+        </is>
+      </c>
+      <c r="G7">
+        <v>0.8410124478746281</v>
+      </c>
+      <c r="H7">
+        <v>686095</v>
+      </c>
+      <c r="I7">
+        <v>11</v>
+      </c>
+      <c r="J7">
+        <v>4</v>
+      </c>
+      <c r="K7">
+        <v>7</v>
+      </c>
+      <c r="L7">
+        <v>0.8952070312424085</v>
+      </c>
+      <c r="M7">
+        <v>0.5274883324116374</v>
+      </c>
+      <c r="N7">
+        <v>1.591714515180035</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conditional intensity</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">log_footprint_area</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Footprint area</t>
+        </is>
+      </c>
+      <c r="D8">
+        <v>-0.5866286129292264</v>
+      </c>
+      <c r="E8">
+        <v>0.5561992904299969</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">weighted R-squared</t>
+        </is>
+      </c>
+      <c r="G8">
+        <v>0.3113439102768608</v>
+      </c>
+      <c r="H8">
+        <v>134863</v>
+      </c>
+      <c r="I8">
+        <v>11</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>11</v>
+      </c>
+      <c r="L8">
+        <v>0.5356380750647078</v>
+      </c>
+      <c r="M8">
+        <v>0.3733317415601784</v>
+      </c>
+      <c r="N8">
+        <v>0.7974759711184671</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conditional intensity</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">compactness</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Planform compactness</t>
+        </is>
+      </c>
+      <c r="D9">
+        <v>0.13201554504897564</v>
+      </c>
+      <c r="E9">
+        <v>1.1411260579898188</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">weighted R-squared</t>
+        </is>
+      </c>
+      <c r="G9">
+        <v>0.3113439102768608</v>
+      </c>
+      <c r="H9">
+        <v>134863</v>
+      </c>
+      <c r="I9">
+        <v>11</v>
+      </c>
+      <c r="J9">
+        <v>11</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
+      <c r="L9">
+        <v>1.1118452796633032</v>
+      </c>
+      <c r="M9">
+        <v>1.0004313793102084</v>
+      </c>
+      <c r="N9">
+        <v>1.296584390166494</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conditional intensity</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">log_elongation</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Planform elongation</t>
+        </is>
+      </c>
+      <c r="D10">
+        <v>0.09100045914824642</v>
+      </c>
+      <c r="E10">
+        <v>1.095269508149424</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">weighted R-squared</t>
+        </is>
+      </c>
+      <c r="G10">
+        <v>0.3113439102768608</v>
+      </c>
+      <c r="H10">
+        <v>134863</v>
+      </c>
+      <c r="I10">
+        <v>11</v>
+      </c>
+      <c r="J10">
+        <v>10</v>
+      </c>
+      <c r="K10">
+        <v>1</v>
+      </c>
+      <c r="L10">
+        <v>1.0451197266867276</v>
+      </c>
+      <c r="M10">
+        <v>0.9577881879970743</v>
+      </c>
+      <c r="N10">
+        <v>1.1383324609423342</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conditional intensity</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cardinal_alignment</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cardinal-axis alignment</t>
+        </is>
+      </c>
+      <c r="D11">
+        <v>-0.022854327185099367</v>
+      </c>
+      <c r="E11">
+        <v>0.9774048547197216</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">weighted R-squared</t>
+        </is>
+      </c>
+      <c r="G11">
+        <v>0.3113439102768608</v>
+      </c>
+      <c r="H11">
+        <v>134863</v>
+      </c>
+      <c r="I11">
+        <v>11</v>
+      </c>
+      <c r="J11">
+        <v>6</v>
+      </c>
+      <c r="K11">
+        <v>5</v>
+      </c>
+      <c r="L11">
+        <v>1.0029781439315653</v>
+      </c>
+      <c r="M11">
+        <v>0.967188370252759</v>
+      </c>
+      <c r="N11">
+        <v>1.0473746909555517</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conditional intensity</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">log_local_building_density</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Local building density</t>
+        </is>
+      </c>
+      <c r="D12">
+        <v>-0.0549235701820393</v>
+      </c>
+      <c r="E12">
+        <v>0.9465574904055695</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">weighted R-squared</t>
+        </is>
+      </c>
+      <c r="G12">
+        <v>0.3113439102768608</v>
+      </c>
+      <c r="H12">
+        <v>134863</v>
+      </c>
+      <c r="I12">
+        <v>11</v>
+      </c>
+      <c r="J12">
+        <v>3</v>
+      </c>
+      <c r="K12">
+        <v>8</v>
+      </c>
+      <c r="L12">
+        <v>0.9294178346050193</v>
+      </c>
+      <c r="M12">
+        <v>0.7647534051841322</v>
+      </c>
+      <c r="N12">
+        <v>1.0827209446858814</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conditional intensity</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">log_local_footprint_coverage</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Local footprint coverage</t>
+        </is>
+      </c>
+      <c r="D13">
+        <v>-0.00917413343818258</v>
+      </c>
+      <c r="E13">
+        <v>0.9908678205288663</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">weighted R-squared</t>
+        </is>
+      </c>
+      <c r="G13">
+        <v>0.3113439102768608</v>
+      </c>
+      <c r="H13">
+        <v>134863</v>
+      </c>
+      <c r="I13">
+        <v>11</v>
+      </c>
+      <c r="J13">
+        <v>5</v>
+      </c>
+      <c r="K13">
+        <v>6</v>
+      </c>
+      <c r="L13">
+        <v>0.9915696822703602</v>
+      </c>
+      <c r="M13">
+        <v>0.8505872311071927</v>
+      </c>
+      <c r="N13">
+        <v>1.2258136899009018</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:N13"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:S13"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">city_key</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">City</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">building_count</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">pv_positive_buildings</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">valid_planform_count</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">valid_planform_share_pct</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">eligible_grid_building_count</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">eligible_grid_building_share_pct</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">model_eligible_count</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">model_eligible_share_pct</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">model_eligible_pv_positive</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">sampled_negative_count</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">median_footprint_area_m2</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">median_compactness</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">median_elongation</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">median_local_building_density_per_km2</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">median_local_footprint_coverage_pct</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">pv_positive_intensity_gt_1_count</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">pv_positive_intensity_gt_1_share_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vienna</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vienna</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>261797</v>
+      </c>
+      <c r="D2">
+        <v>16620</v>
+      </c>
+      <c r="E2">
+        <v>261788</v>
+      </c>
+      <c r="F2">
+        <v>99.9965622218742</v>
+      </c>
+      <c r="G2">
+        <v>260153</v>
+      </c>
+      <c r="H2">
+        <v>99.3720325290206</v>
+      </c>
+      <c r="I2">
+        <v>260144</v>
+      </c>
+      <c r="J2">
+        <v>99.36859475089476</v>
+      </c>
+      <c r="K2">
+        <v>16535</v>
+      </c>
+      <c r="L2">
+        <v>50000</v>
+      </c>
+      <c r="M2">
+        <v>79.28494033593091</v>
+      </c>
+      <c r="N2">
+        <v>0.7087599346717166</v>
+      </c>
+      <c r="O2">
+        <v>1.4085305675532127</v>
+      </c>
+      <c r="P2">
+        <v>1024.0</v>
+      </c>
+      <c r="Q2">
+        <v>18.278524010150694</v>
+      </c>
+      <c r="R2">
+        <v>285</v>
+      </c>
+      <c r="S2">
+        <v>1.7236165709101905</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bratislava</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bratislava</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>101906</v>
+      </c>
+      <c r="D3">
+        <v>2686</v>
+      </c>
+      <c r="E3">
+        <v>101906</v>
+      </c>
+      <c r="F3">
+        <v>100.0</v>
+      </c>
+      <c r="G3">
+        <v>100302</v>
+      </c>
+      <c r="H3">
+        <v>98.42600043177046</v>
+      </c>
+      <c r="I3">
+        <v>100302</v>
+      </c>
+      <c r="J3">
+        <v>98.42600043177046</v>
+      </c>
+      <c r="K3">
+        <v>2650</v>
+      </c>
+      <c r="L3">
+        <v>50000</v>
+      </c>
+      <c r="M3">
+        <v>66.79622946939156</v>
+      </c>
+      <c r="N3">
+        <v>0.7107285843516895</v>
+      </c>
+      <c r="O3">
+        <v>1.5525396613462903</v>
+      </c>
+      <c r="P3">
+        <v>820.0</v>
+      </c>
+      <c r="Q3">
+        <v>12.910822987265288</v>
+      </c>
+      <c r="R3">
+        <v>28</v>
+      </c>
+      <c r="S3">
+        <v>1.0566037735849056</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">singapore</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Singapore</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>282069</v>
+      </c>
+      <c r="D4">
+        <v>12737</v>
+      </c>
+      <c r="E4">
+        <v>282069</v>
+      </c>
+      <c r="F4">
+        <v>100.0</v>
+      </c>
+      <c r="G4">
+        <v>277896</v>
+      </c>
+      <c r="H4">
+        <v>98.52057475298597</v>
+      </c>
+      <c r="I4">
+        <v>277896</v>
+      </c>
+      <c r="J4">
+        <v>98.52057475298597</v>
+      </c>
+      <c r="K4">
+        <v>12655</v>
+      </c>
+      <c r="L4">
+        <v>50000</v>
+      </c>
+      <c r="M4">
+        <v>103.62932749048456</v>
+      </c>
+      <c r="N4">
+        <v>0.6845321113048614</v>
+      </c>
+      <c r="O4">
+        <v>1.7914229270051387</v>
+      </c>
+      <c r="P4">
+        <v>558.0</v>
+      </c>
+      <c r="Q4">
+        <v>24.218140390696828</v>
+      </c>
+      <c r="R4">
+        <v>456</v>
+      </c>
+      <c r="S4">
+        <v>3.603318846305808</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">johorbahru</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Johor Bahru</t>
+        </is>
+      </c>
+      <c r="C5">
+        <v>563858</v>
+      </c>
+      <c r="D5">
+        <v>4874</v>
+      </c>
+      <c r="E5">
+        <v>563858</v>
+      </c>
+      <c r="F5">
+        <v>100.0</v>
+      </c>
+      <c r="G5">
+        <v>559503</v>
+      </c>
+      <c r="H5">
+        <v>99.22764242060944</v>
+      </c>
+      <c r="I5">
+        <v>559503</v>
+      </c>
+      <c r="J5">
+        <v>99.22764242060944</v>
+      </c>
+      <c r="K5">
+        <v>4859</v>
+      </c>
+      <c r="L5">
+        <v>50000</v>
+      </c>
+      <c r="M5">
+        <v>86.20194489935645</v>
+      </c>
+      <c r="N5">
+        <v>0.7047667755728934</v>
+      </c>
+      <c r="O5">
+        <v>1.735843040985329</v>
+      </c>
+      <c r="P5">
+        <v>1285.0</v>
+      </c>
+      <c r="Q5">
+        <v>22.006063905430544</v>
+      </c>
+      <c r="R5">
+        <v>96</v>
+      </c>
+      <c r="S5">
+        <v>1.9757151677299856</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sandiego</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">San Diego</t>
+        </is>
+      </c>
+      <c r="C6">
+        <v>414749</v>
+      </c>
+      <c r="D6">
+        <v>59463</v>
+      </c>
+      <c r="E6">
+        <v>414749</v>
+      </c>
+      <c r="F6">
+        <v>100.0</v>
+      </c>
+      <c r="G6">
+        <v>411467</v>
+      </c>
+      <c r="H6">
+        <v>99.20867801971796</v>
+      </c>
+      <c r="I6">
+        <v>411467</v>
+      </c>
+      <c r="J6">
+        <v>99.20867801971796</v>
+      </c>
+      <c r="K6">
+        <v>59155</v>
+      </c>
+      <c r="L6">
+        <v>50000</v>
+      </c>
+      <c r="M6">
+        <v>183.1166950897109</v>
+      </c>
+      <c r="N6">
+        <v>0.6324638068744597</v>
+      </c>
+      <c r="O6">
+        <v>1.4025726253954829</v>
+      </c>
+      <c r="P6">
+        <v>910.0</v>
+      </c>
+      <c r="Q6">
+        <v>19.03687403850928</v>
+      </c>
+      <c r="R6">
+        <v>278</v>
+      </c>
+      <c r="S6">
+        <v>0.4699518214859268</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tijuana</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tijuana</t>
+        </is>
+      </c>
+      <c r="C7">
+        <v>1438885</v>
+      </c>
+      <c r="D7">
+        <v>4456</v>
+      </c>
+      <c r="E7">
+        <v>1438829</v>
+      </c>
+      <c r="F7">
+        <v>99.99610809758946</v>
+      </c>
+      <c r="G7">
+        <v>1438265</v>
+      </c>
+      <c r="H7">
+        <v>99.95691108045466</v>
+      </c>
+      <c r="I7">
+        <v>1438209</v>
+      </c>
+      <c r="J7">
+        <v>99.95301917804412</v>
+      </c>
+      <c r="K7">
+        <v>4450</v>
+      </c>
+      <c r="L7">
+        <v>50000</v>
+      </c>
+      <c r="M7">
+        <v>27.76414453403737</v>
+      </c>
+      <c r="N7">
+        <v>0.7112605179751194</v>
+      </c>
+      <c r="O7">
+        <v>1.5036084449036151</v>
+      </c>
+      <c r="P7">
+        <v>5397.0</v>
+      </c>
+      <c r="Q7">
+        <v>24.162013525207836</v>
+      </c>
+      <c r="R7">
+        <v>279</v>
+      </c>
+      <c r="S7">
+        <v>6.269662921348315</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">elpaso</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El Paso</t>
+        </is>
+      </c>
+      <c r="C8">
+        <v>316020</v>
+      </c>
+      <c r="D8">
+        <v>10953</v>
+      </c>
+      <c r="E8">
+        <v>316020</v>
+      </c>
+      <c r="F8">
+        <v>100.0</v>
+      </c>
+      <c r="G8">
+        <v>314308</v>
+      </c>
+      <c r="H8">
+        <v>99.45826213530788</v>
+      </c>
+      <c r="I8">
+        <v>314308</v>
+      </c>
+      <c r="J8">
+        <v>99.45826213530788</v>
+      </c>
+      <c r="K8">
+        <v>10879</v>
+      </c>
+      <c r="L8">
+        <v>50000</v>
+      </c>
+      <c r="M8">
+        <v>166.91523007584988</v>
+      </c>
+      <c r="N8">
+        <v>0.7133364258106123</v>
+      </c>
+      <c r="O8">
+        <v>1.3524410095872297</v>
+      </c>
+      <c r="P8">
+        <v>913.0</v>
+      </c>
+      <c r="Q8">
+        <v>18.08813594344178</v>
+      </c>
+      <c r="R8">
+        <v>39</v>
+      </c>
+      <c r="S8">
+        <v>0.3584888316940895</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juarez</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Juarez</t>
+        </is>
+      </c>
+      <c r="C9">
+        <v>779737</v>
+      </c>
+      <c r="D9">
+        <v>7975</v>
+      </c>
+      <c r="E9">
+        <v>779737</v>
+      </c>
+      <c r="F9">
+        <v>100.0</v>
+      </c>
+      <c r="G9">
+        <v>779094</v>
+      </c>
+      <c r="H9">
+        <v>99.91753629749518</v>
+      </c>
+      <c r="I9">
+        <v>779094</v>
+      </c>
+      <c r="J9">
+        <v>99.91753629749518</v>
+      </c>
+      <c r="K9">
+        <v>7973</v>
+      </c>
+      <c r="L9">
+        <v>50000</v>
+      </c>
+      <c r="M9">
+        <v>51.6432233945728</v>
+      </c>
+      <c r="N9">
+        <v>0.7415677867013897</v>
+      </c>
+      <c r="O9">
+        <v>1.4482368025380934</v>
+      </c>
+      <c r="P9">
+        <v>3078.0</v>
+      </c>
+      <c r="Q9">
+        <v>26.80984663582406</v>
+      </c>
+      <c r="R9">
+        <v>281</v>
+      </c>
+      <c r="S9">
+        <v>3.52439483255989</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hongkong</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hong Kong</t>
+        </is>
+      </c>
+      <c r="C10">
+        <v>413781</v>
+      </c>
+      <c r="D10">
+        <v>12171</v>
+      </c>
+      <c r="E10">
+        <v>413781</v>
+      </c>
+      <c r="F10">
+        <v>100.0</v>
+      </c>
+      <c r="G10">
+        <v>407133</v>
+      </c>
+      <c r="H10">
+        <v>98.3933530055754</v>
+      </c>
+      <c r="I10">
+        <v>407133</v>
+      </c>
+      <c r="J10">
+        <v>98.3933530055754</v>
+      </c>
+      <c r="K10">
+        <v>12102</v>
+      </c>
+      <c r="L10">
+        <v>50000</v>
+      </c>
+      <c r="M10">
+        <v>55.12438833991664</v>
+      </c>
+      <c r="N10">
+        <v>0.6948455918487905</v>
+      </c>
+      <c r="O10">
+        <v>1.635381519191856</v>
+      </c>
+      <c r="P10">
+        <v>1103.0</v>
+      </c>
+      <c r="Q10">
+        <v>14.035319077121422</v>
+      </c>
+      <c r="R10">
+        <v>1324</v>
+      </c>
+      <c r="S10">
+        <v>10.940340439596762</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">shenzhen</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shenzhen</t>
+        </is>
+      </c>
+      <c r="C11">
+        <v>78604</v>
+      </c>
+      <c r="D11">
+        <v>3758</v>
+      </c>
+      <c r="E11">
+        <v>78564</v>
+      </c>
+      <c r="F11">
+        <v>99.94911200447817</v>
+      </c>
+      <c r="G11">
+        <v>65401</v>
+      </c>
+      <c r="H11">
+        <v>83.20314487812325</v>
+      </c>
+      <c r="I11">
+        <v>65379</v>
+      </c>
+      <c r="J11">
+        <v>83.17515648058624</v>
+      </c>
+      <c r="K11">
+        <v>2584</v>
+      </c>
+      <c r="L11">
+        <v>50000</v>
+      </c>
+      <c r="M11">
+        <v>400.5167303907385</v>
+      </c>
+      <c r="N11">
+        <v>0.6649666541857499</v>
+      </c>
+      <c r="O11">
+        <v>1.5187935841488196</v>
+      </c>
+      <c r="P11">
+        <v>168.0</v>
+      </c>
+      <c r="Q11">
+        <v>13.39966177173729</v>
+      </c>
+      <c r="R11">
+        <v>16</v>
+      </c>
+      <c r="S11">
+        <v>0.6191950464396285</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">monaco</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Monaco</t>
+        </is>
+      </c>
+      <c r="C12">
+        <v>1352</v>
+      </c>
+      <c r="D12">
+        <v>34</v>
+      </c>
+      <c r="E12">
+        <v>1345</v>
+      </c>
+      <c r="F12">
+        <v>99.48224852071006</v>
+      </c>
+      <c r="G12">
+        <v>1268</v>
+      </c>
+      <c r="H12">
+        <v>93.78698224852072</v>
+      </c>
+      <c r="I12">
+        <v>1264</v>
+      </c>
+      <c r="J12">
+        <v>93.49112426035504</v>
+      </c>
+      <c r="K12">
+        <v>32</v>
+      </c>
+      <c r="L12">
+        <v>1232</v>
+      </c>
+      <c r="M12">
+        <v>251.07140512287253</v>
+      </c>
+      <c r="N12">
+        <v>0.7061958025270367</v>
+      </c>
+      <c r="O12">
+        <v>1.4887905179667151</v>
+      </c>
+      <c r="P12">
+        <v>341.0</v>
+      </c>
+      <c r="Q12">
+        <v>20.92499326889721</v>
+      </c>
+      <c r="R12">
+        <v>1</v>
+      </c>
+      <c r="S12">
+        <v>3.125</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nice</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nice</t>
+        </is>
+      </c>
+      <c r="C13">
+        <v>56898</v>
+      </c>
+      <c r="D13">
+        <v>991</v>
+      </c>
+      <c r="E13">
+        <v>56889</v>
+      </c>
+      <c r="F13">
+        <v>99.9841822208162</v>
+      </c>
+      <c r="G13">
+        <v>56671</v>
+      </c>
+      <c r="H13">
+        <v>99.60104045836408</v>
+      </c>
+      <c r="I13">
+        <v>56662</v>
+      </c>
+      <c r="J13">
+        <v>99.58522267918028</v>
+      </c>
+      <c r="K13">
+        <v>989</v>
+      </c>
+      <c r="L13">
+        <v>50000</v>
+      </c>
+      <c r="M13">
+        <v>69.76397814023355</v>
+      </c>
+      <c r="N13">
+        <v>0.6775966764573325</v>
+      </c>
+      <c r="O13">
+        <v>1.5884952011828624</v>
+      </c>
+      <c r="P13">
+        <v>959.0</v>
+      </c>
+      <c r="Q13">
+        <v>14.830353081545695</v>
+      </c>
+      <c r="R13">
+        <v>16</v>
+      </c>
+      <c r="S13">
+        <v>1.6177957532861478</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:S13"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:S29"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">city</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">city_key</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">sector</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">system_size_kw</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">cost_per_w_usd</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">import_rate_usd_per_kwh</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">export_low_usd_per_kwh</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">export_mid_usd_per_kwh</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">export_high_usd_per_kwh</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">annual_yield_kwh_per_kw</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">support_fraction</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">fixed_support_usd</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">value_model</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">cost_basis</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">tariff_basis</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">support_basis</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">export_value_display</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">support_display</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">cost_basis_short</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vienna</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vienna</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential</t>
+        </is>
+      </c>
+      <c r="D2">
+        <v>5.0</v>
+      </c>
+      <c r="E2">
+        <v>2.2</v>
+      </c>
+      <c r="F2">
+        <v>0.3132</v>
+      </c>
+      <c r="G2">
+        <v>0.216</v>
+      </c>
+      <c r="H2">
+        <v>0.216</v>
+      </c>
+      <c r="I2">
+        <v>0.216</v>
+      </c>
+      <c r="J2">
+        <v>1150.0</v>
+      </c>
+      <c r="K2">
+        <v>0.2</v>
+      </c>
+      <c r="L2">
+        <v>0.0</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">self_consumption_plus_export</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current 5 kW residential anchor</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current audited city export input</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current central capital-support assumption</t>
+        </is>
+      </c>
+      <c r="Q2">
+        <v>0.216</v>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20\%</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vienna</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vienna</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Small commercial</t>
+        </is>
+      </c>
+      <c r="D3">
+        <v>100.0</v>
+      </c>
+      <c r="E3">
+        <v>1.4184397163120568</v>
+      </c>
+      <c r="F3">
+        <v>0.232</v>
+      </c>
+      <c r="G3">
+        <v>0.216</v>
+      </c>
+      <c r="H3">
+        <v>0.216</v>
+      </c>
+      <c r="I3">
+        <v>0.216</v>
+      </c>
+      <c r="J3">
+        <v>1150.0</v>
+      </c>
+      <c r="K3">
+        <v>0.2</v>
+      </c>
+      <c r="L3">
+        <v>0.0</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">self_consumption_plus_export</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current residential anchor times 0.6447; direct Austria 2024 ratio</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current audited city export input</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current central capital-support assumption</t>
+        </is>
+      </c>
+      <c r="Q3">
+        <v>0.216</v>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20\%</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Direct Austrian ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bratislava</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bratislava</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential</t>
+        </is>
+      </c>
+      <c r="D4">
+        <v>5.0</v>
+      </c>
+      <c r="E4">
+        <v>1.9</v>
+      </c>
+      <c r="F4">
+        <v>0.2088</v>
+      </c>
+      <c r="G4">
+        <v>0.173</v>
+      </c>
+      <c r="H4">
+        <v>0.173</v>
+      </c>
+      <c r="I4">
+        <v>0.173</v>
+      </c>
+      <c r="J4">
+        <v>1150.0</v>
+      </c>
+      <c r="K4">
+        <v>0.1</v>
+      </c>
+      <c r="L4">
+        <v>0.0</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">self_consumption_plus_export</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current 5 kW residential anchor</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current audited city export input</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current central capital-support assumption</t>
+        </is>
+      </c>
+      <c r="Q4">
+        <v>0.173</v>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10\%</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bratislava</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bratislava</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Small commercial</t>
+        </is>
+      </c>
+      <c r="D5">
+        <v>100.0</v>
+      </c>
+      <c r="E5">
+        <v>1.52</v>
+      </c>
+      <c r="F5">
+        <v>0.1856</v>
+      </c>
+      <c r="G5">
+        <v>0.173</v>
+      </c>
+      <c r="H5">
+        <v>0.173</v>
+      </c>
+      <c r="I5">
+        <v>0.173</v>
+      </c>
+      <c r="J5">
+        <v>1150.0</v>
+      </c>
+      <c r="K5">
+        <v>0.1</v>
+      </c>
+      <c r="L5">
+        <v>0.0</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">self_consumption_plus_export</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current residential anchor times 0.8000; pooled transferred ratio</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current audited city export input</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current central capital-support assumption</t>
+        </is>
+      </c>
+      <c r="Q5">
+        <v>0.173</v>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10\%</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transferred 0.80 ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Singapore</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">singapore</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential</t>
+        </is>
+      </c>
+      <c r="D6">
+        <v>5.0</v>
+      </c>
+      <c r="E6">
+        <v>1.2</v>
+      </c>
+      <c r="F6">
+        <v>0.2315</v>
+      </c>
+      <c r="G6">
+        <v>0.219</v>
+      </c>
+      <c r="H6">
+        <v>0.219</v>
+      </c>
+      <c r="I6">
+        <v>0.219</v>
+      </c>
+      <c r="J6">
+        <v>1450.0</v>
+      </c>
+      <c r="K6">
+        <v>0.0</v>
+      </c>
+      <c r="L6">
+        <v>0.0</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">self_consumption_plus_export</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current 5 kW residential anchor</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current audited city export input</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EMA states no general generation subsidy</t>
+        </is>
+      </c>
+      <c r="Q6">
+        <v>0.219</v>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Singapore</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">singapore</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Small commercial</t>
+        </is>
+      </c>
+      <c r="D7">
+        <v>100.0</v>
+      </c>
+      <c r="E7">
+        <v>0.96</v>
+      </c>
+      <c r="F7">
+        <v>0.2125</v>
+      </c>
+      <c r="G7">
+        <v>0.078</v>
+      </c>
+      <c r="H7">
+        <v>0.146</v>
+      </c>
+      <c r="I7">
+        <v>0.214</v>
+      </c>
+      <c r="J7">
+        <v>1450.0</v>
+      </c>
+      <c r="K7">
+        <v>0.0</v>
+      </c>
+      <c r="L7">
+        <v>0.0</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">self_consumption_plus_export</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current residential anchor times 0.8000; pooled transferred ratio</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EMA contestable-consumer wholesale-price range</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EMA states no general generation subsidy</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.078--0.214</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transferred 0.80 ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Johor Bahru</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">johorbahru</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential</t>
+        </is>
+      </c>
+      <c r="D8">
+        <v>5.0</v>
+      </c>
+      <c r="E8">
+        <v>1.0</v>
+      </c>
+      <c r="F8">
+        <v>0.1289</v>
+      </c>
+      <c r="G8">
+        <v>0.1289</v>
+      </c>
+      <c r="H8">
+        <v>0.1289</v>
+      </c>
+      <c r="I8">
+        <v>0.1289</v>
+      </c>
+      <c r="J8">
+        <v>1450.0</v>
+      </c>
+      <c r="K8">
+        <v>0.0</v>
+      </c>
+      <c r="L8">
+        <v>0.0</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">self_consumption_plus_export</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current 5 kW residential anchor</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NEM Rakyat one-for-one tariff offset</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NEM value represented through bill credits, not CAPEX reduction</t>
+        </is>
+      </c>
+      <c r="Q8">
+        <v>0.129</v>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Johor Bahru</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">johorbahru</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Small commercial</t>
+        </is>
+      </c>
+      <c r="D9">
+        <v>100.0</v>
+      </c>
+      <c r="E9">
+        <v>0.7939068100358422</v>
+      </c>
+      <c r="F9">
+        <v>0.1274</v>
+      </c>
+      <c r="G9">
+        <v>0.07</v>
+      </c>
+      <c r="H9">
+        <v>0.07</v>
+      </c>
+      <c r="I9">
+        <v>0.07</v>
+      </c>
+      <c r="J9">
+        <v>1450.0</v>
+      </c>
+      <c r="K9">
+        <v>0.0</v>
+      </c>
+      <c r="L9">
+        <v>0.0</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">self_consumption_plus_export</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current residential anchor times 0.7939; Malaysia 2019 ratio applied to current anchor</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NOVA System Marginal Price proxy</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NEM value represented through bill credits, not CAPEX reduction</t>
+        </is>
+      </c>
+      <c r="Q9">
+        <v>0.070</v>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Malaysia sector ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">San Diego</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sandiego</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential</t>
+        </is>
+      </c>
+      <c r="D10">
+        <v>5.0</v>
+      </c>
+      <c r="E10">
+        <v>2.6</v>
+      </c>
+      <c r="F10">
+        <v>0.3197</v>
+      </c>
+      <c r="G10">
+        <v>0.03</v>
+      </c>
+      <c r="H10">
+        <v>0.03</v>
+      </c>
+      <c r="I10">
+        <v>0.03</v>
+      </c>
+      <c r="J10">
+        <v>1650.0</v>
+      </c>
+      <c r="K10">
+        <v>0.3</v>
+      </c>
+      <c r="L10">
+        <v>0.0</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">self_consumption_plus_export</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current 5 kW residential anchor</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current audited city export input</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">study-vintage US 30% credit realization scenario</t>
+        </is>
+      </c>
+      <c r="Q10">
+        <v>0.030</v>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30\%</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">San Diego</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sandiego</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Small commercial</t>
+        </is>
+      </c>
+      <c r="D11">
+        <v>100.0</v>
+      </c>
+      <c r="E11">
+        <v>2.1047619047619044</v>
+      </c>
+      <c r="F11">
+        <v>0.2443</v>
+      </c>
+      <c r="G11">
+        <v>0.03</v>
+      </c>
+      <c r="H11">
+        <v>0.03</v>
+      </c>
+      <c r="I11">
+        <v>0.03</v>
+      </c>
+      <c r="J11">
+        <v>1650.0</v>
+      </c>
+      <c r="K11">
+        <v>0.3</v>
+      </c>
+      <c r="L11">
+        <v>0.0</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">self_consumption_plus_export</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current residential anchor times 0.8095; California 2023 observed ratio</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current audited city export input</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">study-vintage US 30% credit realization scenario</t>
+        </is>
+      </c>
+      <c r="Q11">
+        <v>0.030</v>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30\%</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">California sector ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tijuana</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tijuana</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential</t>
+        </is>
+      </c>
+      <c r="D12">
+        <v>5.0</v>
+      </c>
+      <c r="E12">
+        <v>1.6</v>
+      </c>
+      <c r="F12">
+        <v>0.1221</v>
+      </c>
+      <c r="G12">
+        <v>0.1221</v>
+      </c>
+      <c r="H12">
+        <v>0.1221</v>
+      </c>
+      <c r="I12">
+        <v>0.1221</v>
+      </c>
+      <c r="J12">
+        <v>1650.0</v>
+      </c>
+      <c r="K12">
+        <v>0.1</v>
+      </c>
+      <c r="L12">
+        <v>0.0</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">self_consumption_plus_export</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current 5 kW residential anchor</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mexico monthly net-metering tariff-class proxy</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current central capital-support assumption</t>
+        </is>
+      </c>
+      <c r="Q12">
+        <v>0.122</v>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10\%</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tijuana</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tijuana</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Small commercial</t>
+        </is>
+      </c>
+      <c r="D13">
+        <v>100.0</v>
+      </c>
+      <c r="E13">
+        <v>1.2800000000000002</v>
+      </c>
+      <c r="F13">
+        <v>0.0547</v>
+      </c>
+      <c r="G13">
+        <v>0.0547</v>
+      </c>
+      <c r="H13">
+        <v>0.0547</v>
+      </c>
+      <c r="I13">
+        <v>0.0547</v>
+      </c>
+      <c r="J13">
+        <v>1650.0</v>
+      </c>
+      <c r="K13">
+        <v>0.1</v>
+      </c>
+      <c r="L13">
+        <v>0.0</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">self_consumption_plus_export</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current residential anchor times 0.8000; pooled transferred ratio</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mexico monthly net-metering tariff-class proxy</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current central capital-support assumption</t>
+        </is>
+      </c>
+      <c r="Q13">
+        <v>0.055</v>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10\%</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transferred 0.80 ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detroit</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">detroit</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential</t>
+        </is>
+      </c>
+      <c r="D14">
+        <v>5.0</v>
+      </c>
+      <c r="E14">
+        <v>3.77</v>
+      </c>
+      <c r="F14">
+        <v>0.1859120833333333</v>
+      </c>
+      <c r="G14">
+        <v>0.1045420833333333</v>
+      </c>
+      <c r="H14">
+        <v>0.1045420833333333</v>
+      </c>
+      <c r="I14">
+        <v>0.1045420833333333</v>
+      </c>
+      <c r="J14">
+        <v>1200.0</v>
+      </c>
+      <c r="K14">
+        <v>0.3</v>
+      </c>
+      <c r="L14">
+        <v>0.0</v>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">self_consumption_plus_export</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current 5 kW residential anchor</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current audited city export input</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">study-vintage US 30% credit realization scenario</t>
+        </is>
+      </c>
+      <c r="Q14">
+        <v>0.105</v>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30\%</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detroit</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">detroit</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Small commercial</t>
+        </is>
+      </c>
+      <c r="D15">
+        <v>100.0</v>
+      </c>
+      <c r="E15">
+        <v>3.0607920792079204</v>
+      </c>
+      <c r="F15">
+        <v>0.1401</v>
+      </c>
+      <c r="G15">
+        <v>0.1045420833333333</v>
+      </c>
+      <c r="H15">
+        <v>0.1045420833333333</v>
+      </c>
+      <c r="I15">
+        <v>0.1045420833333333</v>
+      </c>
+      <c r="J15">
+        <v>1200.0</v>
+      </c>
+      <c r="K15">
+        <v>0.3</v>
+      </c>
+      <c r="L15">
+        <v>0.0</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">self_consumption_plus_export</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current residential anchor times 0.8119; United States 2023 observed ratio</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024 Michigan commercial average energy rate; demand charges excluded</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">study-vintage US 30% credit realization scenario</t>
+        </is>
+      </c>
+      <c r="Q15">
+        <v>0.105</v>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30\%</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">US sector ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Windsor</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">windsor</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential</t>
+        </is>
+      </c>
+      <c r="D16">
+        <v>5.0</v>
+      </c>
+      <c r="E16">
+        <v>2.5722318757798392</v>
+      </c>
+      <c r="F16">
+        <v>0.1154949502930087</v>
+      </c>
+      <c r="G16">
+        <v>0.1154949502930087</v>
+      </c>
+      <c r="H16">
+        <v>0.1154949502930087</v>
+      </c>
+      <c r="I16">
+        <v>0.1154949502930087</v>
+      </c>
+      <c r="J16">
+        <v>1200.0</v>
+      </c>
+      <c r="K16">
+        <v>0.0</v>
+      </c>
+      <c r="L16">
+        <v>3650.167907723755</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">self_consumption_plus_export</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current 5 kW residential anchor</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ontario net-metering variable bill-credit proxy</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">realized residential grant from audited central scenario</t>
+        </is>
+      </c>
+      <c r="Q16">
+        <v>0.115</v>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">US\$3,650 fixed</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Windsor</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">windsor</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Small commercial</t>
+        </is>
+      </c>
+      <c r="D17">
+        <v>100.0</v>
+      </c>
+      <c r="E17">
+        <v>2.157355766783091</v>
+      </c>
+      <c r="F17">
+        <v>0.1154949502930087</v>
+      </c>
+      <c r="G17">
+        <v>0.1154949502930087</v>
+      </c>
+      <c r="H17">
+        <v>0.1154949502930087</v>
+      </c>
+      <c r="I17">
+        <v>0.1154949502930087</v>
+      </c>
+      <c r="J17">
+        <v>1200.0</v>
+      </c>
+      <c r="K17">
+        <v>0.0</v>
+      </c>
+      <c r="L17">
+        <v>0.0</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">self_consumption_plus_export</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current residential anchor times 0.8387; Canada 2024 midpoint ratio</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ontario net-metering variable bill-credit proxy</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">residential grant excluded from commercial scenario</t>
+        </is>
+      </c>
+      <c r="Q17">
+        <v>0.115</v>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Canada sector ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El Paso</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">elpaso</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential</t>
+        </is>
+      </c>
+      <c r="D18">
+        <v>5.0</v>
+      </c>
+      <c r="E18">
+        <v>2.34</v>
+      </c>
+      <c r="F18">
+        <v>0.1494</v>
+      </c>
+      <c r="G18">
+        <v>0.02</v>
+      </c>
+      <c r="H18">
+        <v>0.02</v>
+      </c>
+      <c r="I18">
+        <v>0.02</v>
+      </c>
+      <c r="J18">
+        <v>1750.0</v>
+      </c>
+      <c r="K18">
+        <v>0.3</v>
+      </c>
+      <c r="L18">
+        <v>0.0</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">self_consumption_plus_export</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current 5 kW residential anchor</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current audited city export input</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">study-vintage US 30% credit realization scenario</t>
+        </is>
+      </c>
+      <c r="Q18">
+        <v>0.020</v>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30\%</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El Paso</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">elpaso</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Small commercial</t>
+        </is>
+      </c>
+      <c r="D19">
+        <v>100.0</v>
+      </c>
+      <c r="E19">
+        <v>1.598048780487805</v>
+      </c>
+      <c r="F19">
+        <v>0.0729</v>
+      </c>
+      <c r="G19">
+        <v>0.02</v>
+      </c>
+      <c r="H19">
+        <v>0.02</v>
+      </c>
+      <c r="I19">
+        <v>0.02</v>
+      </c>
+      <c r="J19">
+        <v>1750.0</v>
+      </c>
+      <c r="K19">
+        <v>0.3</v>
+      </c>
+      <c r="L19">
+        <v>0.0</v>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">self_consumption_plus_export</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current residential anchor times 0.6829; Texas 2023 observed ratio</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current audited city export input</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">study-vintage US 30% credit realization scenario</t>
+        </is>
+      </c>
+      <c r="Q19">
+        <v>0.020</v>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30\%</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Texas sector ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ciudad Juarez</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juarez</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential</t>
+        </is>
+      </c>
+      <c r="D20">
+        <v>5.0</v>
+      </c>
+      <c r="E20">
+        <v>1.6</v>
+      </c>
+      <c r="F20">
+        <v>0.1221</v>
+      </c>
+      <c r="G20">
+        <v>0.1221</v>
+      </c>
+      <c r="H20">
+        <v>0.1221</v>
+      </c>
+      <c r="I20">
+        <v>0.1221</v>
+      </c>
+      <c r="J20">
+        <v>1750.0</v>
+      </c>
+      <c r="K20">
+        <v>0.1</v>
+      </c>
+      <c r="L20">
+        <v>0.0</v>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">self_consumption_plus_export</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current 5 kW residential anchor</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mexico monthly net-metering tariff-class proxy</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current central capital-support assumption</t>
+        </is>
+      </c>
+      <c r="Q20">
+        <v>0.122</v>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10\%</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ciudad Juarez</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juarez</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Small commercial</t>
+        </is>
+      </c>
+      <c r="D21">
+        <v>100.0</v>
+      </c>
+      <c r="E21">
+        <v>1.2800000000000002</v>
+      </c>
+      <c r="F21">
+        <v>0.0875</v>
+      </c>
+      <c r="G21">
+        <v>0.0875</v>
+      </c>
+      <c r="H21">
+        <v>0.0875</v>
+      </c>
+      <c r="I21">
+        <v>0.0875</v>
+      </c>
+      <c r="J21">
+        <v>1750.0</v>
+      </c>
+      <c r="K21">
+        <v>0.1</v>
+      </c>
+      <c r="L21">
+        <v>0.0</v>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">self_consumption_plus_export</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current residential anchor times 0.8000; pooled transferred ratio</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mexico monthly net-metering tariff-class proxy</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current central capital-support assumption</t>
+        </is>
+      </c>
+      <c r="Q21">
+        <v>0.087</v>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10\%</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transferred 0.80 ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hong Kong</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hongkong</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential</t>
+        </is>
+      </c>
+      <c r="D22">
+        <v>5.0</v>
+      </c>
+      <c r="E22">
+        <v>2.5</v>
+      </c>
+      <c r="F22">
+        <v>0.1794</v>
+      </c>
+      <c r="G22">
+        <v>0.5128205128205129</v>
+      </c>
+      <c r="H22">
+        <v>0.5128205128205129</v>
+      </c>
+      <c r="I22">
+        <v>0.5128205128205129</v>
+      </c>
+      <c r="J22">
+        <v>1350.0</v>
+      </c>
+      <c r="K22">
+        <v>0.0</v>
+      </c>
+      <c r="L22">
+        <v>0.0</v>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gross_fiT</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current 5 kW residential anchor</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hong Kong gross FiT capacity band</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FiT represented through gross generation revenue</t>
+        </is>
+      </c>
+      <c r="Q22">
+        <v>0.513</v>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gross FiT in value model</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hong Kong</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hongkong</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Small commercial</t>
+        </is>
+      </c>
+      <c r="D23">
+        <v>100.0</v>
+      </c>
+      <c r="E23">
+        <v>2.0</v>
+      </c>
+      <c r="F23">
+        <v>0.1914</v>
+      </c>
+      <c r="G23">
+        <v>0.3846153846153846</v>
+      </c>
+      <c r="H23">
+        <v>0.3846153846153846</v>
+      </c>
+      <c r="I23">
+        <v>0.3846153846153846</v>
+      </c>
+      <c r="J23">
+        <v>1350.0</v>
+      </c>
+      <c r="K23">
+        <v>0.0</v>
+      </c>
+      <c r="L23">
+        <v>0.0</v>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gross_fiT</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current residential anchor times 0.8000; pooled transferred ratio</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hong Kong gross FiT capacity band</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FiT represented through gross generation revenue</t>
+        </is>
+      </c>
+      <c r="Q23">
+        <v>0.385</v>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gross FiT in value model</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transferred 0.80 ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shenzhen</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">shenzhen</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential</t>
+        </is>
+      </c>
+      <c r="D24">
+        <v>5.0</v>
+      </c>
+      <c r="E24">
+        <v>0.6</v>
+      </c>
+      <c r="F24">
+        <v>0.0967</v>
+      </c>
+      <c r="G24">
+        <v>0.07</v>
+      </c>
+      <c r="H24">
+        <v>0.07</v>
+      </c>
+      <c r="I24">
+        <v>0.07</v>
+      </c>
+      <c r="J24">
+        <v>1350.0</v>
+      </c>
+      <c r="K24">
+        <v>0.15</v>
+      </c>
+      <c r="L24">
+        <v>0.0</v>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">self_consumption_plus_export</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current 5 kW residential anchor</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current audited city export input</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current central capital-support assumption</t>
+        </is>
+      </c>
+      <c r="Q24">
+        <v>0.070</v>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15\%</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shenzhen</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">shenzhen</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Small commercial</t>
+        </is>
+      </c>
+      <c r="D25">
+        <v>100.0</v>
+      </c>
+      <c r="E25">
+        <v>0.5823529411764705</v>
+      </c>
+      <c r="F25">
+        <v>0.1145</v>
+      </c>
+      <c r="G25">
+        <v>0.07</v>
+      </c>
+      <c r="H25">
+        <v>0.07</v>
+      </c>
+      <c r="I25">
+        <v>0.07</v>
+      </c>
+      <c r="J25">
+        <v>1350.0</v>
+      </c>
+      <c r="K25">
+        <v>0.15</v>
+      </c>
+      <c r="L25">
+        <v>0.0</v>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">self_consumption_plus_export</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current residential anchor times 0.9706; China 2024 direct ratio</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current audited city export input</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current central capital-support assumption</t>
+        </is>
+      </c>
+      <c r="Q25">
+        <v>0.070</v>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15\%</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">China sector ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Monaco</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">monaco</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential</t>
+        </is>
+      </c>
+      <c r="D26">
+        <v>5.0</v>
+      </c>
+      <c r="E26">
+        <v>2.6</v>
+      </c>
+      <c r="F26">
+        <v>0.2279</v>
+      </c>
+      <c r="G26">
+        <v>0.173</v>
+      </c>
+      <c r="H26">
+        <v>0.173</v>
+      </c>
+      <c r="I26">
+        <v>0.173</v>
+      </c>
+      <c r="J26">
+        <v>1500.0</v>
+      </c>
+      <c r="K26">
+        <v>0.2</v>
+      </c>
+      <c r="L26">
+        <v>0.0</v>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">self_consumption_plus_export</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current 5 kW residential anchor</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current audited city export input</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current central capital-support assumption</t>
+        </is>
+      </c>
+      <c r="Q26">
+        <v>0.173</v>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20\%</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Monaco</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">monaco</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Small commercial</t>
+        </is>
+      </c>
+      <c r="D27">
+        <v>100.0</v>
+      </c>
+      <c r="E27">
+        <v>2.08</v>
+      </c>
+      <c r="F27">
+        <v>0.2279</v>
+      </c>
+      <c r="G27">
+        <v>0.173</v>
+      </c>
+      <c r="H27">
+        <v>0.173</v>
+      </c>
+      <c r="I27">
+        <v>0.173</v>
+      </c>
+      <c r="J27">
+        <v>1500.0</v>
+      </c>
+      <c r="K27">
+        <v>0.2</v>
+      </c>
+      <c r="L27">
+        <v>0.0</v>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">self_consumption_plus_export</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current residential anchor times 0.8000; pooled transferred ratio</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current audited city export input</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current central capital-support assumption</t>
+        </is>
+      </c>
+      <c r="Q27">
+        <v>0.173</v>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20\%</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transferred 0.80 ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nice</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nice</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential</t>
+        </is>
+      </c>
+      <c r="D28">
+        <v>5.0</v>
+      </c>
+      <c r="E28">
+        <v>2.2</v>
+      </c>
+      <c r="F28">
+        <v>0.225</v>
+      </c>
+      <c r="G28">
+        <v>0.173</v>
+      </c>
+      <c r="H28">
+        <v>0.173</v>
+      </c>
+      <c r="I28">
+        <v>0.173</v>
+      </c>
+      <c r="J28">
+        <v>1500.0</v>
+      </c>
+      <c r="K28">
+        <v>0.2</v>
+      </c>
+      <c r="L28">
+        <v>0.0</v>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">self_consumption_plus_export</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current 5 kW residential anchor</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current audited city export input</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current central capital-support assumption</t>
+        </is>
+      </c>
+      <c r="Q28">
+        <v>0.173</v>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20\%</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nice</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nice</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Small commercial</t>
+        </is>
+      </c>
+      <c r="D29">
+        <v>100.0</v>
+      </c>
+      <c r="E29">
+        <v>1.7600000000000002</v>
+      </c>
+      <c r="F29">
+        <v>0.1856</v>
+      </c>
+      <c r="G29">
+        <v>0.173</v>
+      </c>
+      <c r="H29">
+        <v>0.173</v>
+      </c>
+      <c r="I29">
+        <v>0.173</v>
+      </c>
+      <c r="J29">
+        <v>1500.0</v>
+      </c>
+      <c r="K29">
+        <v>0.2</v>
+      </c>
+      <c r="L29">
+        <v>0.0</v>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">self_consumption_plus_export</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current residential anchor times 0.8000; pooled transferred ratio</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current audited city export input</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">current central capital-support assumption</t>
+        </is>
+      </c>
+      <c r="Q29">
+        <v>0.173</v>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20\%</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transferred 0.80 ratio</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:S29"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:I37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -7812,7 +11649,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15"/>

</xml_diff>